<commit_message>
add event activity status
</commit_message>
<xml_diff>
--- a/data/applications.xlsx
+++ b/data/applications.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -439,9 +439,69 @@
         <v>30.03.2026 12:48:32</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>nalan</v>
+      </c>
+      <c r="B3" t="str">
+        <v>kara</v>
+      </c>
+      <c r="C3" t="str">
+        <v>ornek@gmail.com</v>
+      </c>
+      <c r="D3" t="str">
+        <v>05555555555</v>
+      </c>
+      <c r="E3" t="str">
+        <v>sosyal-medya</v>
+      </c>
+      <c r="F3" t="str">
+        <v>30.03.2026 13:16:59</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>nalan</v>
+      </c>
+      <c r="B4" t="str">
+        <v>kara</v>
+      </c>
+      <c r="C4" t="str">
+        <v>example@gmail.com</v>
+      </c>
+      <c r="D4" t="str">
+        <v>05555555555</v>
+      </c>
+      <c r="E4" t="str">
+        <v>egitim</v>
+      </c>
+      <c r="F4" t="str">
+        <v>30.03.2026 13:23:37</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>emircan</v>
+      </c>
+      <c r="B5" t="str">
+        <v>kural</v>
+      </c>
+      <c r="C5" t="str">
+        <v>emircank@gmail.com</v>
+      </c>
+      <c r="D5" t="str">
+        <v>05555555555</v>
+      </c>
+      <c r="E5" t="str">
+        <v>tasarim</v>
+      </c>
+      <c r="F5" t="str">
+        <v>30.03.2026 14:44:49</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>